<commit_message>
Working update with Volume objective integrated
</commit_message>
<xml_diff>
--- a/Data_v4.xlsx
+++ b/Data_v4.xlsx
@@ -1,21 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29512"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://upatrasgr-my.sharepoint.com/personal/mead6828_upatras_gr/Documents/Patch_Strength_Prediction/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="267" documentId="11_4F0ECDF259EC9F3A877A2395395BDA16F642DD1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31E4A178-4275-4492-820B-AD4DB115E495}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="3870" yWindow="4005" windowWidth="28800" windowHeight="15435" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Elips0" sheetId="1" r:id="rId1"/>
     <sheet name="Elips1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="76">
   <si>
     <t>Specimen_ID</t>
   </si>
@@ -68,6 +90,9 @@
     <t>Predicted_Strength_Mean</t>
   </si>
   <si>
+    <t>Expected Improvement</t>
+  </si>
+  <si>
     <t>Specimen_1</t>
   </si>
   <si>
@@ -209,20 +234,44 @@
     <t>Specimen_48</t>
   </si>
   <si>
+    <t>Specimen_49</t>
+  </si>
+  <si>
+    <t>Specimen_50</t>
+  </si>
+  <si>
+    <t>Specimen_51</t>
+  </si>
+  <si>
+    <t>Specimen_52</t>
+  </si>
+  <si>
+    <t>Specimen_53</t>
+  </si>
+  <si>
+    <t>Specimen_54</t>
+  </si>
+  <si>
+    <t>Specimen_55</t>
+  </si>
+  <si>
+    <t>Specimen_56</t>
+  </si>
+  <si>
+    <t>Specimen_57</t>
+  </si>
+  <si>
     <t>Specimen_42</t>
   </si>
   <si>
-    <t>Specimen_49</t>
-  </si>
-  <si>
-    <t>Specimen_50</t>
+    <t>Specimen_58</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,18 +282,38 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -274,17 +343,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -572,11 +653,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q48"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:X57"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="17" max="17" width="16.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:24">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -628,10 +713,19 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:17">
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+    </row>
+    <row r="2" spans="1:24">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>7.7</v>
@@ -672,22 +766,19 @@
       <c r="N2">
         <v>0</v>
       </c>
-      <c r="O2">
-        <v>6889.387025616274</v>
-      </c>
       <c r="P2">
         <v>49.77</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>7.1</v>
       </c>
       <c r="C3">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="D3">
         <v>11.4</v>
@@ -708,7 +799,7 @@
         <v>7.1</v>
       </c>
       <c r="J3">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="K3">
         <v>11.4</v>
@@ -722,16 +813,13 @@
       <c r="N3">
         <v>0</v>
       </c>
-      <c r="O3">
-        <v>5339.01105106971</v>
-      </c>
       <c r="P3">
         <v>45.69</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:24">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>6.8</v>
@@ -772,16 +860,13 @@
       <c r="N4">
         <v>0</v>
       </c>
-      <c r="O4">
-        <v>4311.77308519892</v>
-      </c>
       <c r="P4">
         <v>52.67</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:24">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5">
         <v>6.5</v>
@@ -822,16 +907,13 @@
       <c r="N5">
         <v>0</v>
       </c>
-      <c r="O5">
-        <v>3666.050131180073</v>
-      </c>
       <c r="P5">
         <v>41.62</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:24">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>6.3</v>
@@ -872,16 +954,13 @@
       <c r="N6">
         <v>0</v>
       </c>
-      <c r="O6">
-        <v>3201.911232538717</v>
-      </c>
       <c r="P6">
         <v>38.58</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:24">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7">
         <v>6.2</v>
@@ -893,7 +972,7 @@
         <v>8.5</v>
       </c>
       <c r="E7">
-        <v>9.699999999999999</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="F7">
         <v>10.9</v>
@@ -914,7 +993,7 @@
         <v>8.5</v>
       </c>
       <c r="L7">
-        <v>9.699999999999999</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="M7">
         <v>10.9</v>
@@ -922,16 +1001,13 @@
       <c r="N7">
         <v>0</v>
       </c>
-      <c r="O7">
-        <v>2873.237809120153</v>
-      </c>
       <c r="P7">
         <v>41.61</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:24">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8">
         <v>6.1</v>
@@ -940,10 +1016,10 @@
         <v>7.1</v>
       </c>
       <c r="D8">
-        <v>8.199999999999999</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="E8">
-        <v>9.199999999999999</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="F8">
         <v>10.3</v>
@@ -961,10 +1037,10 @@
         <v>7.1</v>
       </c>
       <c r="K8">
-        <v>8.199999999999999</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="L8">
-        <v>9.199999999999999</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="M8">
         <v>10.3</v>
@@ -972,16 +1048,13 @@
       <c r="N8">
         <v>0</v>
       </c>
-      <c r="O8">
-        <v>2630.267033291519</v>
-      </c>
       <c r="P8">
         <v>40.6</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:24">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9">
         <v>6.2</v>
@@ -990,7 +1063,7 @@
         <v>9</v>
       </c>
       <c r="D9">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="E9">
         <v>13</v>
@@ -1022,16 +1095,13 @@
       <c r="N9">
         <v>0</v>
       </c>
-      <c r="O9">
-        <v>5142.347350954989</v>
-      </c>
       <c r="P9">
         <v>64.47</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:24">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10">
         <v>6.2</v>
@@ -1072,19 +1142,16 @@
       <c r="N10">
         <v>0</v>
       </c>
-      <c r="O10">
-        <v>4760.769507249974</v>
-      </c>
       <c r="P10">
         <v>53.6</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:24">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11">
-        <v>8.300000000000001</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="C11">
         <v>15.7</v>
@@ -1117,30 +1184,27 @@
         <v>18.2</v>
       </c>
       <c r="M11">
-        <v>33.8</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="N11">
         <v>0</v>
-      </c>
-      <c r="O11">
-        <v>18642.08514269569</v>
       </c>
       <c r="P11">
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:24">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12">
-        <v>8.300000000000001</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="C12">
         <v>14.3</v>
       </c>
       <c r="D12">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="E12">
         <v>25</v>
@@ -1149,13 +1213,13 @@
         <v>30.4</v>
       </c>
       <c r="G12">
-        <v>35.8</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="H12">
         <v>5</v>
       </c>
       <c r="I12">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="J12">
         <v>15.8</v>
@@ -1172,16 +1236,13 @@
       <c r="N12">
         <v>0</v>
       </c>
-      <c r="O12">
-        <v>18676.76832559132</v>
-      </c>
       <c r="P12">
-        <v>73.18000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17">
+        <v>73.180000000000007</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13">
         <v>6.3</v>
@@ -1190,7 +1251,7 @@
         <v>7.5</v>
       </c>
       <c r="D13">
-        <v>8.800000000000001</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="E13">
         <v>10</v>
@@ -1222,16 +1283,13 @@
       <c r="N13">
         <v>0</v>
       </c>
-      <c r="O13">
-        <v>3250.543086816288</v>
-      </c>
       <c r="P13">
         <v>49.65</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:24">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>6.3</v>
@@ -1249,7 +1307,7 @@
         <v>15.3</v>
       </c>
       <c r="G14">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="H14">
         <v>5</v>
@@ -1272,16 +1330,13 @@
       <c r="N14">
         <v>0</v>
       </c>
-      <c r="O14">
-        <v>5259.340261374673</v>
-      </c>
       <c r="P14">
         <v>55.9</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:24">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>8.4</v>
@@ -1311,7 +1366,7 @@
         <v>12.9</v>
       </c>
       <c r="K15">
-        <v>16.9</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="L15">
         <v>20.8</v>
@@ -1322,16 +1377,13 @@
       <c r="N15">
         <v>0</v>
       </c>
-      <c r="O15">
-        <v>11966.89190420117</v>
-      </c>
       <c r="P15">
         <v>58.5</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:24">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16">
         <v>8.4</v>
@@ -1349,7 +1401,7 @@
         <v>27.9</v>
       </c>
       <c r="G16">
-        <v>32.8</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="H16">
         <v>5</v>
@@ -1372,16 +1424,13 @@
       <c r="N16">
         <v>0</v>
       </c>
-      <c r="O16">
-        <v>16034.94023133459</v>
-      </c>
       <c r="P16">
         <v>71.53</v>
       </c>
     </row>
     <row r="17" spans="1:16">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>6</v>
@@ -1422,16 +1471,13 @@
       <c r="N17">
         <v>0</v>
       </c>
-      <c r="O17">
-        <v>2513.274122871835</v>
-      </c>
       <c r="P17">
         <v>71.23</v>
       </c>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18">
         <v>7</v>
@@ -1472,16 +1518,13 @@
       <c r="N18">
         <v>0</v>
       </c>
-      <c r="O18">
-        <v>4963.716392671873</v>
-      </c>
       <c r="P18">
         <v>71.2</v>
       </c>
     </row>
     <row r="19" spans="1:16">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>8</v>
@@ -1522,16 +1565,13 @@
       <c r="N19">
         <v>0</v>
       </c>
-      <c r="O19">
-        <v>8293.804605477053</v>
-      </c>
       <c r="P19">
-        <v>71.31999999999999</v>
+        <v>71.319999999999993</v>
       </c>
     </row>
     <row r="20" spans="1:16">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B20">
         <v>9</v>
@@ -1572,16 +1612,13 @@
       <c r="N20">
         <v>0</v>
       </c>
-      <c r="O20">
-        <v>12503.53876128738</v>
-      </c>
       <c r="P20">
-        <v>71.40000000000001</v>
+        <v>71.400000000000006</v>
       </c>
     </row>
     <row r="21" spans="1:16">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>10</v>
@@ -1622,16 +1659,13 @@
       <c r="N21">
         <v>0</v>
       </c>
-      <c r="O21">
-        <v>17592.91886010284</v>
-      </c>
       <c r="P21">
         <v>71.5</v>
       </c>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B22">
         <v>7</v>
@@ -1672,16 +1706,13 @@
       <c r="N22">
         <v>0</v>
       </c>
-      <c r="O22">
-        <v>3223.274062583127</v>
-      </c>
       <c r="P22">
-        <v>71.23999999999999</v>
+        <v>71.239999999999995</v>
       </c>
     </row>
     <row r="23" spans="1:16">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B23">
         <v>7</v>
@@ -1722,16 +1753,13 @@
       <c r="N23">
         <v>0</v>
       </c>
-      <c r="O23">
-        <v>5573.185367468292</v>
-      </c>
       <c r="P23">
         <v>71.27</v>
       </c>
     </row>
     <row r="24" spans="1:16">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B24">
         <v>7</v>
@@ -1772,16 +1800,13 @@
       <c r="N24">
         <v>0</v>
       </c>
-      <c r="O24">
-        <v>6245.486195336509</v>
-      </c>
       <c r="P24">
         <v>71.28</v>
       </c>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B25">
         <v>7</v>
@@ -1822,16 +1847,13 @@
       <c r="N25">
         <v>0</v>
       </c>
-      <c r="O25">
-        <v>5284.158843338032</v>
-      </c>
       <c r="P25">
         <v>52.73</v>
       </c>
     </row>
     <row r="26" spans="1:16">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B26">
         <v>7</v>
@@ -1872,16 +1894,13 @@
       <c r="N26">
         <v>0</v>
       </c>
-      <c r="O26">
-        <v>6088.406562657019</v>
-      </c>
       <c r="P26">
         <v>71.27</v>
       </c>
     </row>
     <row r="27" spans="1:16">
       <c r="A27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B27">
         <v>8</v>
@@ -1922,16 +1941,13 @@
       <c r="N27">
         <v>0</v>
       </c>
-      <c r="O27">
-        <v>3292.389100962103</v>
-      </c>
       <c r="P27">
         <v>71.28</v>
       </c>
     </row>
     <row r="28" spans="1:16">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28">
         <v>8</v>
@@ -1972,16 +1988,13 @@
       <c r="N28">
         <v>0</v>
       </c>
-      <c r="O28">
-        <v>4479.911124019045</v>
-      </c>
       <c r="P28">
         <v>58.69</v>
       </c>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B29">
         <v>5</v>
@@ -2022,16 +2035,13 @@
       <c r="N29">
         <v>0</v>
       </c>
-      <c r="O29">
-        <v>2230.530784048753</v>
-      </c>
       <c r="P29">
-        <v>38.34</v>
+        <v>38.340000000000003</v>
       </c>
     </row>
     <row r="30" spans="1:16">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B30">
         <v>5</v>
@@ -2072,16 +2082,13 @@
       <c r="N30">
         <v>0</v>
       </c>
-      <c r="O30">
-        <v>4209.734155810324</v>
-      </c>
       <c r="P30">
         <v>56.59</v>
       </c>
     </row>
     <row r="31" spans="1:16">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B31">
         <v>5</v>
@@ -2122,16 +2129,13 @@
       <c r="N31">
         <v>0</v>
       </c>
-      <c r="O31">
-        <v>6880.087911361647</v>
-      </c>
       <c r="P31">
         <v>69.42</v>
       </c>
     </row>
     <row r="32" spans="1:16">
       <c r="A32" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B32">
         <v>5</v>
@@ -2172,16 +2176,13 @@
       <c r="N32">
         <v>0</v>
       </c>
-      <c r="O32">
-        <v>10241.59205070273</v>
-      </c>
       <c r="P32">
-        <v>69.51000000000001</v>
+        <v>69.510000000000005</v>
       </c>
     </row>
     <row r="33" spans="1:17">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B33">
         <v>5</v>
@@ -2222,16 +2223,13 @@
       <c r="N33">
         <v>0</v>
       </c>
-      <c r="O33">
-        <v>14294.24657383356</v>
-      </c>
       <c r="P33">
         <v>69.58</v>
       </c>
     </row>
     <row r="34" spans="1:17">
       <c r="A34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B34">
         <v>5</v>
@@ -2272,16 +2270,13 @@
       <c r="N34">
         <v>0</v>
       </c>
-      <c r="O34">
-        <v>7809.999336824227</v>
-      </c>
       <c r="P34">
         <v>54.39</v>
       </c>
     </row>
     <row r="35" spans="1:17">
       <c r="A35" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B35">
         <v>5</v>
@@ -2322,16 +2317,13 @@
       <c r="N35">
         <v>0</v>
       </c>
-      <c r="O35">
-        <v>9343.096551776045</v>
-      </c>
       <c r="P35">
         <v>69.45</v>
       </c>
     </row>
     <row r="36" spans="1:17">
       <c r="A36" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B36">
         <v>5</v>
@@ -2372,16 +2364,13 @@
       <c r="N36">
         <v>0</v>
       </c>
-      <c r="O36">
-        <v>11127.52117901505</v>
-      </c>
       <c r="P36">
-        <v>69.51000000000001</v>
+        <v>69.510000000000005</v>
       </c>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B37">
         <v>5</v>
@@ -2422,16 +2411,13 @@
       <c r="N37">
         <v>0</v>
       </c>
-      <c r="O37">
-        <v>5623.45084992573</v>
-      </c>
       <c r="P37">
         <v>42.27</v>
       </c>
     </row>
     <row r="38" spans="1:17">
       <c r="A38" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B38">
         <v>5</v>
@@ -2472,16 +2458,13 @@
       <c r="N38">
         <v>0</v>
       </c>
-      <c r="O38">
-        <v>6930.353393819083</v>
-      </c>
       <c r="P38">
         <v>62.51</v>
       </c>
     </row>
     <row r="39" spans="1:17">
       <c r="A39" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B39">
         <v>5</v>
@@ -2522,16 +2505,13 @@
       <c r="N39">
         <v>0</v>
       </c>
-      <c r="O39">
-        <v>8796.45943005142</v>
-      </c>
       <c r="P39">
         <v>63.27</v>
       </c>
     </row>
     <row r="40" spans="1:17">
-      <c r="A40" t="s">
-        <v>55</v>
+      <c r="A40" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="B40">
         <v>8</v>
@@ -2572,19 +2552,16 @@
       <c r="N40">
         <v>0</v>
       </c>
-      <c r="O40">
-        <v>11780.97245096172</v>
-      </c>
       <c r="P40">
         <v>71.55</v>
       </c>
       <c r="Q40">
-        <v>162.6550903</v>
+        <v>162.65509030000001</v>
       </c>
     </row>
     <row r="41" spans="1:17">
-      <c r="A41" t="s">
-        <v>56</v>
+      <c r="A41" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="B41">
         <v>13</v>
@@ -2625,19 +2602,16 @@
       <c r="N41">
         <v>0</v>
       </c>
-      <c r="O41">
-        <v>13169.55640384841</v>
-      </c>
       <c r="P41">
         <v>55.94</v>
       </c>
       <c r="Q41">
-        <v>159.4312133789062</v>
+        <v>159.43121337890619</v>
       </c>
     </row>
     <row r="42" spans="1:17">
-      <c r="A42" t="s">
-        <v>57</v>
+      <c r="A42" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="B42">
         <v>15</v>
@@ -2679,18 +2653,18 @@
         <v>0</v>
       </c>
       <c r="O42">
-        <v>25000.79433726757</v>
+        <v>2500.079433726758</v>
       </c>
       <c r="P42">
-        <v>71.76000000000001</v>
+        <v>71.760000000000005</v>
       </c>
       <c r="Q42">
         <v>178.8307189941406</v>
       </c>
     </row>
     <row r="43" spans="1:17">
-      <c r="A43" t="s">
-        <v>58</v>
+      <c r="A43" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="B43">
         <v>13</v>
@@ -2732,118 +2706,112 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <v>19546.98949063569</v>
+        <v>1954.698949063569</v>
       </c>
       <c r="P43">
         <v>71.67</v>
       </c>
       <c r="Q43">
-        <v>150.7803802490234</v>
+        <v>150.78038024902341</v>
       </c>
     </row>
     <row r="44" spans="1:17">
-      <c r="A44" t="s">
-        <v>59</v>
-      </c>
-      <c r="B44">
+      <c r="A44" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" s="2">
         <v>14</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="2">
         <v>18</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="2">
         <v>25</v>
       </c>
-      <c r="E44">
+      <c r="E44" s="2">
         <v>28</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="2">
         <v>32</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="2">
         <v>33</v>
       </c>
-      <c r="H44">
+      <c r="H44" s="2">
         <v>13</v>
       </c>
-      <c r="I44">
+      <c r="I44" s="2">
         <v>17</v>
       </c>
-      <c r="J44">
+      <c r="J44" s="2">
         <v>24</v>
       </c>
-      <c r="K44">
+      <c r="K44" s="2">
         <v>27</v>
       </c>
-      <c r="L44">
+      <c r="L44" s="2">
         <v>31</v>
       </c>
-      <c r="M44">
+      <c r="M44" s="2">
         <v>33</v>
       </c>
-      <c r="N44">
-        <v>0</v>
-      </c>
-      <c r="O44">
-        <v>24661.50233067988</v>
-      </c>
-      <c r="P44">
+      <c r="N44" s="2">
+        <v>0</v>
+      </c>
+      <c r="P44" s="2">
         <v>71.7</v>
       </c>
     </row>
     <row r="45" spans="1:17">
-      <c r="A45" t="s">
-        <v>60</v>
-      </c>
-      <c r="B45">
+      <c r="A45" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B45" s="2">
         <v>15</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="2">
         <v>25</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="2">
         <v>30</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="2">
         <v>31</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="2">
         <v>32</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="2">
         <v>33</v>
       </c>
-      <c r="H45">
+      <c r="H45" s="2">
         <v>14</v>
       </c>
-      <c r="I45">
+      <c r="I45" s="2">
         <v>24</v>
       </c>
-      <c r="J45">
+      <c r="J45" s="2">
         <v>29</v>
       </c>
-      <c r="K45">
+      <c r="K45" s="2">
         <v>30</v>
       </c>
-      <c r="L45">
+      <c r="L45" s="2">
         <v>32</v>
       </c>
-      <c r="M45">
+      <c r="M45" s="2">
         <v>33</v>
       </c>
-      <c r="N45">
-        <v>0</v>
-      </c>
-      <c r="O45">
-        <v>29675.48420580919</v>
-      </c>
-      <c r="P45">
+      <c r="N45" s="2">
+        <v>0</v>
+      </c>
+      <c r="P45" s="2">
         <v>50.3</v>
       </c>
     </row>
     <row r="46" spans="1:17">
-      <c r="A46" t="s">
-        <v>61</v>
+      <c r="A46" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="B46">
         <v>5</v>
@@ -2885,18 +2853,18 @@
         <v>0</v>
       </c>
       <c r="O46">
-        <v>5303.00839925957</v>
-      </c>
-      <c r="P46">
+        <v>530.30083992595712</v>
+      </c>
+      <c r="P46" s="2">
         <v>54.2</v>
       </c>
       <c r="Q46">
-        <v>62.69831085205078</v>
+        <v>62.698310852050781</v>
       </c>
     </row>
     <row r="47" spans="1:17">
-      <c r="A47" t="s">
-        <v>62</v>
+      <c r="A47" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="B47">
         <v>5</v>
@@ -2938,9 +2906,9 @@
         <v>0</v>
       </c>
       <c r="O47">
-        <v>2293.362637120549</v>
-      </c>
-      <c r="P47">
+        <v>229.34</v>
+      </c>
+      <c r="P47" s="2">
         <v>71.2</v>
       </c>
       <c r="Q47">
@@ -2948,8 +2916,8 @@
       </c>
     </row>
     <row r="48" spans="1:17">
-      <c r="A48" t="s">
-        <v>63</v>
+      <c r="A48" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="B48">
         <v>5</v>
@@ -2990,27 +2958,490 @@
       <c r="N48">
         <v>0</v>
       </c>
-      <c r="O48">
-        <v>2230.530784048753</v>
-      </c>
-      <c r="P48">
+      <c r="P48" s="2">
         <v>71.2</v>
       </c>
       <c r="Q48">
         <v>61.2</v>
       </c>
     </row>
+    <row r="49" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A49" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B49">
+        <v>21</v>
+      </c>
+      <c r="C49">
+        <v>25</v>
+      </c>
+      <c r="D49">
+        <v>27</v>
+      </c>
+      <c r="E49">
+        <v>28</v>
+      </c>
+      <c r="F49" s="4">
+        <v>29</v>
+      </c>
+      <c r="G49" s="2">
+        <v>35</v>
+      </c>
+      <c r="H49" s="2">
+        <v>5</v>
+      </c>
+      <c r="I49" s="2">
+        <v>12</v>
+      </c>
+      <c r="J49" s="2">
+        <v>14</v>
+      </c>
+      <c r="K49" s="2">
+        <v>20</v>
+      </c>
+      <c r="L49" s="2">
+        <v>22</v>
+      </c>
+      <c r="M49">
+        <v>31</v>
+      </c>
+      <c r="N49">
+        <v>0</v>
+      </c>
+      <c r="P49" s="2">
+        <v>57.3</v>
+      </c>
+      <c r="Q49">
+        <v>64.001168318171622</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18">
+      <c r="A50" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B50">
+        <v>15</v>
+      </c>
+      <c r="C50">
+        <v>22</v>
+      </c>
+      <c r="D50">
+        <v>25</v>
+      </c>
+      <c r="E50">
+        <v>26</v>
+      </c>
+      <c r="F50" s="2">
+        <v>32</v>
+      </c>
+      <c r="G50" s="2">
+        <v>35</v>
+      </c>
+      <c r="H50" s="2">
+        <v>6</v>
+      </c>
+      <c r="I50" s="4">
+        <v>7</v>
+      </c>
+      <c r="J50" s="2">
+        <v>17</v>
+      </c>
+      <c r="K50" s="2">
+        <v>21</v>
+      </c>
+      <c r="L50" s="4">
+        <v>22</v>
+      </c>
+      <c r="M50">
+        <v>27</v>
+      </c>
+      <c r="N50">
+        <v>0</v>
+      </c>
+      <c r="P50" s="2">
+        <v>71.599999999999994</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18">
+      <c r="A51" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B51">
+        <v>17</v>
+      </c>
+      <c r="C51">
+        <v>21</v>
+      </c>
+      <c r="D51">
+        <v>22</v>
+      </c>
+      <c r="E51">
+        <v>27</v>
+      </c>
+      <c r="F51">
+        <v>29</v>
+      </c>
+      <c r="G51">
+        <v>34</v>
+      </c>
+      <c r="H51">
+        <v>7</v>
+      </c>
+      <c r="I51">
+        <v>11</v>
+      </c>
+      <c r="J51">
+        <v>16</v>
+      </c>
+      <c r="K51">
+        <v>17</v>
+      </c>
+      <c r="L51">
+        <v>21</v>
+      </c>
+      <c r="M51">
+        <v>25</v>
+      </c>
+      <c r="N51">
+        <v>0</v>
+      </c>
+      <c r="P51" s="2">
+        <v>71.599999999999994</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18">
+      <c r="A52" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B52">
+        <v>5</v>
+      </c>
+      <c r="C52">
+        <v>11</v>
+      </c>
+      <c r="D52">
+        <v>20</v>
+      </c>
+      <c r="E52">
+        <v>23</v>
+      </c>
+      <c r="F52">
+        <v>27</v>
+      </c>
+      <c r="G52">
+        <v>31</v>
+      </c>
+      <c r="H52">
+        <v>5</v>
+      </c>
+      <c r="I52">
+        <v>10</v>
+      </c>
+      <c r="J52">
+        <v>16</v>
+      </c>
+      <c r="K52">
+        <v>21</v>
+      </c>
+      <c r="L52">
+        <v>25</v>
+      </c>
+      <c r="M52">
+        <v>28</v>
+      </c>
+      <c r="N52">
+        <v>0</v>
+      </c>
+      <c r="P52">
+        <v>71.5</v>
+      </c>
+      <c r="Q52">
+        <v>73.209999999999994</v>
+      </c>
+      <c r="R52">
+        <v>0.12180000000000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18">
+      <c r="A53" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B53">
+        <v>7</v>
+      </c>
+      <c r="C53">
+        <v>9</v>
+      </c>
+      <c r="D53">
+        <v>10</v>
+      </c>
+      <c r="E53">
+        <v>11</v>
+      </c>
+      <c r="F53">
+        <v>33</v>
+      </c>
+      <c r="G53">
+        <v>34</v>
+      </c>
+      <c r="H53">
+        <v>5</v>
+      </c>
+      <c r="I53">
+        <v>9</v>
+      </c>
+      <c r="J53">
+        <v>10</v>
+      </c>
+      <c r="K53">
+        <v>11</v>
+      </c>
+      <c r="L53">
+        <v>18</v>
+      </c>
+      <c r="M53">
+        <v>34</v>
+      </c>
+      <c r="N53">
+        <v>0</v>
+      </c>
+      <c r="P53">
+        <v>57.5</v>
+      </c>
+      <c r="Q53">
+        <v>70.92</v>
+      </c>
+      <c r="R53">
+        <v>0.11799999999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18">
+      <c r="A54" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B54">
+        <v>6</v>
+      </c>
+      <c r="C54">
+        <v>13</v>
+      </c>
+      <c r="D54">
+        <v>16</v>
+      </c>
+      <c r="E54">
+        <v>19</v>
+      </c>
+      <c r="F54">
+        <v>24</v>
+      </c>
+      <c r="G54">
+        <v>29</v>
+      </c>
+      <c r="H54">
+        <v>5</v>
+      </c>
+      <c r="I54">
+        <v>11</v>
+      </c>
+      <c r="J54">
+        <v>14</v>
+      </c>
+      <c r="K54">
+        <v>17</v>
+      </c>
+      <c r="L54">
+        <v>22</v>
+      </c>
+      <c r="M54">
+        <v>25</v>
+      </c>
+      <c r="N54">
+        <v>0</v>
+      </c>
+      <c r="P54">
+        <v>71.400000000000006</v>
+      </c>
+      <c r="Q54">
+        <v>72.95</v>
+      </c>
+      <c r="R54">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18">
+      <c r="A55" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B55">
+        <v>6</v>
+      </c>
+      <c r="C55">
+        <v>7</v>
+      </c>
+      <c r="D55">
+        <v>8</v>
+      </c>
+      <c r="E55">
+        <v>18</v>
+      </c>
+      <c r="F55">
+        <v>24</v>
+      </c>
+      <c r="G55">
+        <v>27</v>
+      </c>
+      <c r="H55">
+        <v>5</v>
+      </c>
+      <c r="I55">
+        <v>7</v>
+      </c>
+      <c r="J55">
+        <v>8</v>
+      </c>
+      <c r="K55">
+        <v>17</v>
+      </c>
+      <c r="L55">
+        <v>23</v>
+      </c>
+      <c r="M55">
+        <v>25</v>
+      </c>
+      <c r="N55">
+        <v>0</v>
+      </c>
+      <c r="P55" s="5">
+        <v>53.8</v>
+      </c>
+      <c r="Q55">
+        <v>71.73</v>
+      </c>
+      <c r="R55">
+        <v>0.126</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18">
+      <c r="A56" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B56">
+        <v>8</v>
+      </c>
+      <c r="C56">
+        <v>9</v>
+      </c>
+      <c r="D56">
+        <v>10</v>
+      </c>
+      <c r="E56">
+        <v>13</v>
+      </c>
+      <c r="F56">
+        <v>20</v>
+      </c>
+      <c r="G56">
+        <v>30</v>
+      </c>
+      <c r="H56">
+        <v>8</v>
+      </c>
+      <c r="I56">
+        <v>9</v>
+      </c>
+      <c r="J56">
+        <v>10</v>
+      </c>
+      <c r="K56">
+        <v>11</v>
+      </c>
+      <c r="L56">
+        <v>19</v>
+      </c>
+      <c r="M56">
+        <v>29</v>
+      </c>
+      <c r="N56">
+        <v>0</v>
+      </c>
+      <c r="P56" s="5">
+        <v>71.3</v>
+      </c>
+      <c r="Q56">
+        <v>69.7</v>
+      </c>
+      <c r="R56">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18">
+      <c r="A57" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B57">
+        <v>12</v>
+      </c>
+      <c r="C57">
+        <v>16</v>
+      </c>
+      <c r="D57">
+        <v>21</v>
+      </c>
+      <c r="E57">
+        <v>22</v>
+      </c>
+      <c r="F57">
+        <v>26</v>
+      </c>
+      <c r="G57">
+        <v>35</v>
+      </c>
+      <c r="H57">
+        <v>8</v>
+      </c>
+      <c r="I57">
+        <v>14</v>
+      </c>
+      <c r="J57">
+        <v>17</v>
+      </c>
+      <c r="K57">
+        <v>22</v>
+      </c>
+      <c r="L57">
+        <v>24</v>
+      </c>
+      <c r="M57">
+        <v>35</v>
+      </c>
+      <c r="N57">
+        <v>0</v>
+      </c>
+      <c r="P57" s="5">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="Q57">
+        <v>71.63</v>
+      </c>
+      <c r="R57">
+        <v>0.11</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q38"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Z46"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3062,10 +3493,21 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:17">
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+    </row>
+    <row r="2" spans="1:26">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>7.7</v>
@@ -3106,16 +3548,13 @@
       <c r="N2">
         <v>1</v>
       </c>
-      <c r="O2">
-        <v>4277.655388980935</v>
-      </c>
       <c r="P2">
         <v>59.02</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>7.1</v>
@@ -3124,10 +3563,10 @@
         <v>7.1</v>
       </c>
       <c r="D3">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="E3">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="F3">
         <v>12.3</v>
@@ -3145,7 +3584,7 @@
         <v>7.1</v>
       </c>
       <c r="K3">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="L3">
         <v>10.8</v>
@@ -3156,16 +3595,13 @@
       <c r="N3">
         <v>1</v>
       </c>
-      <c r="O3">
-        <v>3399.266083037228</v>
-      </c>
       <c r="P3">
         <v>57.46</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>6.8</v>
@@ -3198,7 +3634,7 @@
         <v>8.5</v>
       </c>
       <c r="L4">
-        <v>9.800000000000001</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="M4">
         <v>11</v>
@@ -3206,16 +3642,13 @@
       <c r="N4">
         <v>1</v>
       </c>
-      <c r="O4">
-        <v>2848.733386422153</v>
-      </c>
       <c r="P4">
         <v>58.23</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5">
         <v>6.8</v>
@@ -3248,7 +3681,7 @@
         <v>8.5</v>
       </c>
       <c r="L5">
-        <v>9.800000000000001</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="M5">
         <v>11</v>
@@ -3256,16 +3689,13 @@
       <c r="N5">
         <v>1</v>
       </c>
-      <c r="O5">
-        <v>2848.733386422153</v>
-      </c>
       <c r="P5">
         <v>58.23</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>6.3</v>
@@ -3306,16 +3736,13 @@
       <c r="N6">
         <v>1</v>
       </c>
-      <c r="O6">
-        <v>2251.139631856302</v>
-      </c>
       <c r="P6">
         <v>64.75</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7">
         <v>6.2</v>
@@ -3333,7 +3760,7 @@
         <v>9</v>
       </c>
       <c r="G7">
-        <v>9.800000000000001</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="H7">
         <v>5</v>
@@ -3348,7 +3775,7 @@
         <v>7.3</v>
       </c>
       <c r="L7">
-        <v>8.199999999999999</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="M7">
         <v>9</v>
@@ -3356,16 +3783,13 @@
       <c r="N7">
         <v>1</v>
       </c>
-      <c r="O7">
-        <v>2073.388319516192</v>
-      </c>
       <c r="P7">
         <v>50.68</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8">
         <v>6.1</v>
@@ -3383,7 +3807,7 @@
         <v>8.6</v>
       </c>
       <c r="G8">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="H8">
         <v>5</v>
@@ -3406,16 +3830,13 @@
       <c r="N8">
         <v>1</v>
       </c>
-      <c r="O8">
-        <v>1943.703374776005</v>
-      </c>
       <c r="P8">
         <v>64.75</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:26">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9">
         <v>6.2</v>
@@ -3433,7 +3854,7 @@
         <v>9</v>
       </c>
       <c r="G9">
-        <v>9.800000000000001</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -3448,7 +3869,7 @@
         <v>7.3</v>
       </c>
       <c r="L9">
-        <v>8.199999999999999</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="M9">
         <v>9</v>
@@ -3456,16 +3877,13 @@
       <c r="N9">
         <v>1</v>
       </c>
-      <c r="O9">
-        <v>2073.388319516192</v>
-      </c>
       <c r="P9">
         <v>50.68</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:26">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10">
         <v>6.1</v>
@@ -3483,7 +3901,7 @@
         <v>8.6</v>
       </c>
       <c r="G10">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="H10">
         <v>5</v>
@@ -3506,16 +3924,13 @@
       <c r="N10">
         <v>1</v>
       </c>
-      <c r="O10">
-        <v>1947.536117813384</v>
-      </c>
       <c r="P10">
         <v>64.75</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:26">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>6.3</v>
@@ -3524,7 +3939,7 @@
         <v>7.5</v>
       </c>
       <c r="D11">
-        <v>8.800000000000001</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -3556,16 +3971,13 @@
       <c r="N11">
         <v>1</v>
       </c>
-      <c r="O11">
-        <v>2288.021929609446</v>
-      </c>
       <c r="P11">
         <v>76.66</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:26">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12">
         <v>6.3</v>
@@ -3595,7 +4007,7 @@
         <v>8.1</v>
       </c>
       <c r="K12">
-        <v>9.699999999999999</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="L12">
         <v>11.3</v>
@@ -3606,16 +4018,13 @@
       <c r="N12">
         <v>1</v>
       </c>
-      <c r="O12">
-        <v>3691.685527233366</v>
-      </c>
       <c r="P12">
         <v>71.22</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:26">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13">
         <v>6.2</v>
@@ -3624,7 +4033,7 @@
         <v>7.8</v>
       </c>
       <c r="D13">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="E13">
         <v>10.9</v>
@@ -3656,16 +4065,13 @@
       <c r="N13">
         <v>1</v>
       </c>
-      <c r="O13">
-        <v>3633.880222407314</v>
-      </c>
       <c r="P13">
-        <v>73.06999999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17">
+        <v>73.069999999999993</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>6.2</v>
@@ -3698,7 +4104,7 @@
         <v>8.1</v>
       </c>
       <c r="L14">
-        <v>9.199999999999999</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="M14">
         <v>10.3</v>
@@ -3706,19 +4112,16 @@
       <c r="N14">
         <v>1</v>
       </c>
-      <c r="O14">
-        <v>2493.230761741932</v>
-      </c>
       <c r="P14">
         <v>37.53</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:26">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15">
-        <v>8.300000000000001</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="C15">
         <v>12.4</v>
@@ -3745,7 +4148,7 @@
         <v>13.2</v>
       </c>
       <c r="K15">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="L15">
         <v>21.5</v>
@@ -3756,19 +4159,16 @@
       <c r="N15">
         <v>1</v>
       </c>
-      <c r="O15">
-        <v>12600.04848760565</v>
-      </c>
       <c r="P15">
         <v>76.63</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:26">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16">
-        <v>8.300000000000001</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="C16">
         <v>9.1</v>
@@ -3798,24 +4198,21 @@
         <v>13.2</v>
       </c>
       <c r="L16">
-        <v>16.1</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="M16">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="N16">
         <v>1</v>
       </c>
-      <c r="O16">
-        <v>7024.475509720633</v>
-      </c>
       <c r="P16">
-        <v>73.73999999999999</v>
+        <v>73.739999999999995</v>
       </c>
     </row>
     <row r="17" spans="1:16">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>8.4</v>
@@ -3830,10 +4227,10 @@
         <v>13</v>
       </c>
       <c r="F17">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="G17">
-        <v>18.4</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="H17">
         <v>5</v>
@@ -3851,21 +4248,18 @@
         <v>14.4</v>
       </c>
       <c r="M17">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="N17">
         <v>1</v>
       </c>
-      <c r="O17">
-        <v>5832.806584360953</v>
-      </c>
       <c r="P17">
         <v>61.64</v>
       </c>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18">
         <v>8.4</v>
@@ -3906,16 +4300,13 @@
       <c r="N18">
         <v>1</v>
       </c>
-      <c r="O18">
-        <v>5770.163226848374</v>
-      </c>
       <c r="P18">
         <v>75.81</v>
       </c>
     </row>
     <row r="19" spans="1:16">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>8.4</v>
@@ -3956,16 +4347,13 @@
       <c r="N19">
         <v>1</v>
       </c>
-      <c r="O19">
-        <v>4883.542948152261</v>
-      </c>
       <c r="P19">
         <v>59.04</v>
       </c>
     </row>
     <row r="20" spans="1:16">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B20">
         <v>7</v>
@@ -4006,16 +4394,13 @@
       <c r="N20">
         <v>1</v>
       </c>
-      <c r="O20">
-        <v>4963.716392671873</v>
-      </c>
       <c r="P20">
         <v>48.7</v>
       </c>
     </row>
     <row r="21" spans="1:16">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>8</v>
@@ -4056,16 +4441,13 @@
       <c r="N21">
         <v>1</v>
       </c>
-      <c r="O21">
-        <v>8293.804605477053</v>
-      </c>
       <c r="P21">
         <v>55.97</v>
       </c>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B22">
         <v>5</v>
@@ -4106,16 +4488,13 @@
       <c r="N22">
         <v>1</v>
       </c>
-      <c r="O22">
-        <v>2230.530784048753</v>
-      </c>
       <c r="P22">
-        <v>38.34</v>
+        <v>38.340000000000003</v>
       </c>
     </row>
     <row r="23" spans="1:16">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B23">
         <v>5</v>
@@ -4156,16 +4535,13 @@
       <c r="N23">
         <v>1</v>
       </c>
-      <c r="O23">
-        <v>4209.734155810324</v>
-      </c>
       <c r="P23">
         <v>56.59</v>
       </c>
     </row>
     <row r="24" spans="1:16">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B24">
         <v>5</v>
@@ -4206,16 +4582,13 @@
       <c r="N24">
         <v>1</v>
       </c>
-      <c r="O24">
-        <v>6880.087911361647</v>
-      </c>
       <c r="P24">
         <v>69.42</v>
       </c>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -4256,16 +4629,13 @@
       <c r="N25">
         <v>1</v>
       </c>
-      <c r="O25">
-        <v>10241.59205070273</v>
-      </c>
       <c r="P25">
-        <v>69.51000000000001</v>
+        <v>69.510000000000005</v>
       </c>
     </row>
     <row r="26" spans="1:16">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B26">
         <v>5</v>
@@ -4306,16 +4676,13 @@
       <c r="N26">
         <v>1</v>
       </c>
-      <c r="O26">
-        <v>14294.24657383356</v>
-      </c>
       <c r="P26">
         <v>69.58</v>
       </c>
     </row>
     <row r="27" spans="1:16">
       <c r="A27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B27">
         <v>5</v>
@@ -4356,16 +4723,13 @@
       <c r="N27">
         <v>1</v>
       </c>
-      <c r="O27">
-        <v>7809.999336824227</v>
-      </c>
       <c r="P27">
         <v>54.39</v>
       </c>
     </row>
     <row r="28" spans="1:16">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28">
         <v>5</v>
@@ -4406,16 +4770,13 @@
       <c r="N28">
         <v>1</v>
       </c>
-      <c r="O28">
-        <v>9343.096551776045</v>
-      </c>
       <c r="P28">
         <v>69.45</v>
       </c>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B29">
         <v>5</v>
@@ -4456,16 +4817,13 @@
       <c r="N29">
         <v>1</v>
       </c>
-      <c r="O29">
-        <v>11127.52117901505</v>
-      </c>
       <c r="P29">
-        <v>69.51000000000001</v>
+        <v>69.510000000000005</v>
       </c>
     </row>
     <row r="30" spans="1:16">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B30">
         <v>5</v>
@@ -4506,16 +4864,13 @@
       <c r="N30">
         <v>1</v>
       </c>
-      <c r="O30">
-        <v>5623.45084992573</v>
-      </c>
       <c r="P30">
         <v>42.27</v>
       </c>
     </row>
     <row r="31" spans="1:16">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B31">
         <v>5</v>
@@ -4556,16 +4911,13 @@
       <c r="N31">
         <v>1</v>
       </c>
-      <c r="O31">
-        <v>6930.353393819083</v>
-      </c>
       <c r="P31">
         <v>62.51</v>
       </c>
     </row>
     <row r="32" spans="1:16">
       <c r="A32" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B32">
         <v>5</v>
@@ -4606,16 +4958,13 @@
       <c r="N32">
         <v>1</v>
       </c>
-      <c r="O32">
-        <v>8796.45943005142</v>
-      </c>
       <c r="P32">
         <v>63.27</v>
       </c>
     </row>
-    <row r="33" spans="1:17">
-      <c r="A33" t="s">
-        <v>64</v>
+    <row r="33" spans="1:18">
+      <c r="A33" s="2" t="s">
+        <v>74</v>
       </c>
       <c r="B33">
         <v>27</v>
@@ -4657,18 +5006,18 @@
         <v>1</v>
       </c>
       <c r="O33">
-        <v>32446.36892627538</v>
+        <v>3244.6368926275381</v>
       </c>
       <c r="P33">
         <v>61.56</v>
       </c>
       <c r="Q33">
-        <v>81.81534576416016</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17">
-      <c r="A34" t="s">
-        <v>59</v>
+        <v>81.815345764160156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18">
+      <c r="A34" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="B34">
         <v>14</v>
@@ -4710,7 +5059,7 @@
         <v>1</v>
       </c>
       <c r="O34">
-        <v>26590.44021998401</v>
+        <v>2659.0440219984011</v>
       </c>
       <c r="P34">
         <v>59</v>
@@ -4719,9 +5068,9 @@
         <v>211.7365417480469</v>
       </c>
     </row>
-    <row r="35" spans="1:17">
-      <c r="A35" t="s">
-        <v>60</v>
+    <row r="35" spans="1:18">
+      <c r="A35" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="B35">
         <v>9</v>
@@ -4763,67 +5112,64 @@
         <v>1</v>
       </c>
       <c r="O35">
-        <v>27507.78527483223</v>
+        <v>2750.7785274832231</v>
       </c>
       <c r="P35">
         <v>71.8</v>
       </c>
       <c r="Q35">
-        <v>209.1623992919922</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17">
-      <c r="A36" t="s">
-        <v>61</v>
-      </c>
-      <c r="B36">
-        <v>7</v>
-      </c>
-      <c r="C36">
-        <v>9</v>
-      </c>
-      <c r="D36">
+        <v>209.16239929199219</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18">
+      <c r="A36" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="2">
+        <v>7</v>
+      </c>
+      <c r="C36" s="2">
+        <v>9</v>
+      </c>
+      <c r="D36" s="2">
         <v>24</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="2">
         <v>30</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="2">
         <v>32</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="2">
         <v>33</v>
       </c>
-      <c r="H36">
-        <v>7</v>
-      </c>
-      <c r="I36">
-        <v>9</v>
-      </c>
-      <c r="J36">
+      <c r="H36" s="2">
+        <v>7</v>
+      </c>
+      <c r="I36" s="2">
+        <v>9</v>
+      </c>
+      <c r="J36" s="2">
         <v>19</v>
       </c>
-      <c r="K36">
+      <c r="K36" s="2">
         <v>25</v>
       </c>
-      <c r="L36">
+      <c r="L36" s="2">
         <v>31</v>
       </c>
-      <c r="M36">
+      <c r="M36" s="2">
         <v>33</v>
       </c>
-      <c r="N36">
+      <c r="N36" s="2">
         <v>1</v>
       </c>
-      <c r="O36">
-        <v>21469.64419463264</v>
-      </c>
-      <c r="P36">
+      <c r="P36" s="2">
         <v>62.5</v>
       </c>
     </row>
-    <row r="37" spans="1:17">
-      <c r="A37" t="s">
+    <row r="37" spans="1:18">
+      <c r="A37" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B37">
@@ -4866,17 +5212,17 @@
         <v>1</v>
       </c>
       <c r="O37">
-        <v>8570.264758992955</v>
-      </c>
-      <c r="P37">
+        <v>857.02647589929552</v>
+      </c>
+      <c r="P37" s="2">
         <v>42.7</v>
       </c>
       <c r="Q37">
-        <v>61.67449569702148</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17">
-      <c r="A38" t="s">
+        <v>61.674495697021477</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18">
+      <c r="A38" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B38">
@@ -4919,7 +5265,7 @@
         <v>1</v>
       </c>
       <c r="O38">
-        <v>2230.530784048753</v>
+        <v>223.05</v>
       </c>
       <c r="P38">
         <v>71.2</v>
@@ -4928,7 +5274,423 @@
         <v>58.28</v>
       </c>
     </row>
+    <row r="39" spans="1:18">
+      <c r="A39" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39">
+        <v>10</v>
+      </c>
+      <c r="C39">
+        <v>13</v>
+      </c>
+      <c r="D39">
+        <v>17</v>
+      </c>
+      <c r="E39">
+        <v>22</v>
+      </c>
+      <c r="F39">
+        <v>31</v>
+      </c>
+      <c r="G39">
+        <v>33</v>
+      </c>
+      <c r="H39">
+        <v>9</v>
+      </c>
+      <c r="I39">
+        <v>13</v>
+      </c>
+      <c r="J39">
+        <v>16</v>
+      </c>
+      <c r="K39">
+        <v>21</v>
+      </c>
+      <c r="L39">
+        <v>24</v>
+      </c>
+      <c r="M39">
+        <v>32</v>
+      </c>
+      <c r="N39">
+        <v>1</v>
+      </c>
+      <c r="P39" s="2">
+        <v>60.2</v>
+      </c>
+      <c r="Q39">
+        <v>58.658827448472017</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18">
+      <c r="A40" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40">
+        <v>11</v>
+      </c>
+      <c r="C40">
+        <v>13</v>
+      </c>
+      <c r="D40">
+        <v>19</v>
+      </c>
+      <c r="E40">
+        <v>22</v>
+      </c>
+      <c r="F40">
+        <v>31</v>
+      </c>
+      <c r="G40">
+        <v>32</v>
+      </c>
+      <c r="H40">
+        <v>9</v>
+      </c>
+      <c r="I40">
+        <v>11</v>
+      </c>
+      <c r="J40">
+        <v>17</v>
+      </c>
+      <c r="K40">
+        <v>20</v>
+      </c>
+      <c r="L40">
+        <v>22</v>
+      </c>
+      <c r="M40">
+        <v>32</v>
+      </c>
+      <c r="N40">
+        <v>1</v>
+      </c>
+      <c r="P40" s="2">
+        <v>57.4</v>
+      </c>
+      <c r="Q40">
+        <v>58.658827087301148</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18">
+      <c r="A41" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B41">
+        <v>10</v>
+      </c>
+      <c r="C41">
+        <v>11</v>
+      </c>
+      <c r="D41">
+        <v>16</v>
+      </c>
+      <c r="E41">
+        <v>22</v>
+      </c>
+      <c r="F41">
+        <v>26</v>
+      </c>
+      <c r="G41">
+        <v>27</v>
+      </c>
+      <c r="H41">
+        <v>9</v>
+      </c>
+      <c r="I41">
+        <v>11</v>
+      </c>
+      <c r="J41">
+        <v>16</v>
+      </c>
+      <c r="K41">
+        <v>18</v>
+      </c>
+      <c r="L41">
+        <v>25</v>
+      </c>
+      <c r="M41">
+        <v>27</v>
+      </c>
+      <c r="N41">
+        <v>1</v>
+      </c>
+      <c r="P41">
+        <v>51.8</v>
+      </c>
+      <c r="Q41">
+        <v>64.02</v>
+      </c>
+      <c r="R41">
+        <v>4.8099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18">
+      <c r="A42" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42">
+        <v>11</v>
+      </c>
+      <c r="C42">
+        <v>14</v>
+      </c>
+      <c r="D42">
+        <v>17</v>
+      </c>
+      <c r="E42">
+        <v>24</v>
+      </c>
+      <c r="F42">
+        <v>28</v>
+      </c>
+      <c r="G42">
+        <v>33</v>
+      </c>
+      <c r="H42">
+        <v>5</v>
+      </c>
+      <c r="I42">
+        <v>12</v>
+      </c>
+      <c r="J42">
+        <v>15</v>
+      </c>
+      <c r="K42">
+        <v>18</v>
+      </c>
+      <c r="L42">
+        <v>27</v>
+      </c>
+      <c r="M42">
+        <v>29</v>
+      </c>
+      <c r="N42">
+        <v>1</v>
+      </c>
+      <c r="P42">
+        <v>63.1</v>
+      </c>
+      <c r="Q42">
+        <v>63.96</v>
+      </c>
+      <c r="R42">
+        <v>4.7699999999999999E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18">
+      <c r="A43" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B43">
+        <v>5</v>
+      </c>
+      <c r="C43">
+        <v>7</v>
+      </c>
+      <c r="D43">
+        <v>13</v>
+      </c>
+      <c r="E43">
+        <v>16</v>
+      </c>
+      <c r="F43">
+        <v>21</v>
+      </c>
+      <c r="G43">
+        <v>26</v>
+      </c>
+      <c r="H43">
+        <v>5</v>
+      </c>
+      <c r="I43">
+        <v>7</v>
+      </c>
+      <c r="J43">
+        <v>13</v>
+      </c>
+      <c r="K43">
+        <v>14</v>
+      </c>
+      <c r="L43">
+        <v>21</v>
+      </c>
+      <c r="M43">
+        <v>23</v>
+      </c>
+      <c r="N43">
+        <v>1</v>
+      </c>
+      <c r="P43">
+        <v>67</v>
+      </c>
+      <c r="Q43">
+        <v>63.8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18">
+      <c r="A44" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B44">
+        <v>6</v>
+      </c>
+      <c r="C44">
+        <v>8</v>
+      </c>
+      <c r="D44">
+        <v>13</v>
+      </c>
+      <c r="E44">
+        <v>22</v>
+      </c>
+      <c r="F44">
+        <v>24</v>
+      </c>
+      <c r="G44">
+        <v>30</v>
+      </c>
+      <c r="H44">
+        <v>5</v>
+      </c>
+      <c r="I44">
+        <v>8</v>
+      </c>
+      <c r="J44">
+        <v>10</v>
+      </c>
+      <c r="K44">
+        <v>18</v>
+      </c>
+      <c r="L44">
+        <v>24</v>
+      </c>
+      <c r="M44">
+        <v>26</v>
+      </c>
+      <c r="N44">
+        <v>1</v>
+      </c>
+      <c r="P44" s="5">
+        <v>71.400000000000006</v>
+      </c>
+      <c r="Q44">
+        <v>72.8</v>
+      </c>
+      <c r="R44">
+        <v>0.14899999999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18">
+      <c r="A45" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B45">
+        <v>5</v>
+      </c>
+      <c r="C45">
+        <v>8</v>
+      </c>
+      <c r="D45">
+        <v>9</v>
+      </c>
+      <c r="E45">
+        <v>13</v>
+      </c>
+      <c r="F45">
+        <v>15</v>
+      </c>
+      <c r="G45">
+        <v>16</v>
+      </c>
+      <c r="H45">
+        <v>5</v>
+      </c>
+      <c r="I45">
+        <v>7</v>
+      </c>
+      <c r="J45">
+        <v>9</v>
+      </c>
+      <c r="K45">
+        <v>11</v>
+      </c>
+      <c r="L45">
+        <v>14</v>
+      </c>
+      <c r="M45">
+        <v>16</v>
+      </c>
+      <c r="N45">
+        <v>1</v>
+      </c>
+      <c r="P45" s="5">
+        <v>71.2</v>
+      </c>
+      <c r="Q45">
+        <v>70.87</v>
+      </c>
+      <c r="R45">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18">
+      <c r="A46" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B46">
+        <v>7</v>
+      </c>
+      <c r="C46">
+        <v>8</v>
+      </c>
+      <c r="D46">
+        <v>12</v>
+      </c>
+      <c r="E46">
+        <v>14</v>
+      </c>
+      <c r="F46">
+        <v>16</v>
+      </c>
+      <c r="G46">
+        <v>17</v>
+      </c>
+      <c r="H46">
+        <v>6</v>
+      </c>
+      <c r="I46">
+        <v>8</v>
+      </c>
+      <c r="J46">
+        <v>9</v>
+      </c>
+      <c r="K46">
+        <v>13</v>
+      </c>
+      <c r="L46">
+        <v>16</v>
+      </c>
+      <c r="M46">
+        <v>17</v>
+      </c>
+      <c r="N46">
+        <v>1</v>
+      </c>
+      <c r="P46" s="5">
+        <v>51.7</v>
+      </c>
+      <c r="Q46">
+        <v>68.39</v>
+      </c>
+      <c r="R46">
+        <v>0.08</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
correct contrain savings. Everything is now correct
</commit_message>
<xml_diff>
--- a/Data_v4.xlsx
+++ b/Data_v4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://upatrasgr-my.sharepoint.com/personal/mead6828_upatras_gr/Documents/Patch_Strength_Prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="977" documentId="11_4F0ECDF259EC9F3A877A2395395BDA16F642DD1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB50A503-7131-4FCB-9C5B-003697822C08}"/>
+  <xr:revisionPtr revIDLastSave="1109" documentId="11_4F0ECDF259EC9F3A877A2395395BDA16F642DD1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B52FBA3-07D0-46F6-A022-1667A9355452}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1305" yWindow="3000" windowWidth="26205" windowHeight="11385" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Elips0" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="100">
   <si>
     <t>Specimen_ID</t>
   </si>
@@ -319,6 +319,18 @@
   </si>
   <si>
     <t>Specimen_76</t>
+  </si>
+  <si>
+    <t>Specimen_77</t>
+  </si>
+  <si>
+    <t>Specimen_78</t>
+  </si>
+  <si>
+    <t>Specimen_79</t>
+  </si>
+  <si>
+    <t>Specimen_80</t>
   </si>
   <si>
     <t>Expected Strength  Improvement</t>
@@ -331,7 +343,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -409,7 +421,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -418,6 +430,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -433,10 +447,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -724,14 +734,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X76"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:X80"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
     <col min="17" max="17" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -795,7 +805,7 @@
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -842,7 +852,7 @@
         <v>49.77</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -889,7 +899,7 @@
         <v>45.69</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -936,7 +946,7 @@
         <v>52.67</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -983,7 +993,7 @@
         <v>41.62</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -1030,7 +1040,7 @@
         <v>38.58</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1077,7 +1087,7 @@
         <v>41.61</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1124,7 +1134,7 @@
         <v>40.6</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1171,7 +1181,7 @@
         <v>64.47</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -1218,7 +1228,7 @@
         <v>53.6</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1265,7 +1275,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1312,7 +1322,7 @@
         <v>73.180000000000007</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -1359,7 +1369,7 @@
         <v>49.65</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -1406,7 +1416,7 @@
         <v>55.9</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -1453,7 +1463,7 @@
         <v>58.5</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -1500,7 +1510,7 @@
         <v>71.53</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -1547,7 +1557,7 @@
         <v>71.23</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -1594,7 +1604,7 @@
         <v>71.2</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -1641,7 +1651,7 @@
         <v>71.319999999999993</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -1688,7 +1698,7 @@
         <v>71.400000000000006</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1735,7 +1745,7 @@
         <v>71.5</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -1782,7 +1792,7 @@
         <v>71.239999999999995</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -1829,7 +1839,7 @@
         <v>71.27</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16">
       <c r="A24" t="s">
         <v>41</v>
       </c>
@@ -1876,7 +1886,7 @@
         <v>71.28</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16">
       <c r="A25" t="s">
         <v>42</v>
       </c>
@@ -1923,7 +1933,7 @@
         <v>52.73</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -1970,7 +1980,7 @@
         <v>71.27</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16">
       <c r="A27" t="s">
         <v>44</v>
       </c>
@@ -2017,7 +2027,7 @@
         <v>71.28</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16">
       <c r="A28" t="s">
         <v>45</v>
       </c>
@@ -2064,7 +2074,7 @@
         <v>58.69</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16">
       <c r="A29" t="s">
         <v>46</v>
       </c>
@@ -2111,7 +2121,7 @@
         <v>38.340000000000003</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16">
       <c r="A30" t="s">
         <v>47</v>
       </c>
@@ -2158,7 +2168,7 @@
         <v>56.59</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -2205,7 +2215,7 @@
         <v>69.42</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16">
       <c r="A32" t="s">
         <v>49</v>
       </c>
@@ -2252,7 +2262,7 @@
         <v>69.510000000000005</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17">
       <c r="A33" t="s">
         <v>50</v>
       </c>
@@ -2299,7 +2309,7 @@
         <v>69.58</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17">
       <c r="A34" t="s">
         <v>51</v>
       </c>
@@ -2346,7 +2356,7 @@
         <v>54.39</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17">
       <c r="A35" t="s">
         <v>52</v>
       </c>
@@ -2393,7 +2403,7 @@
         <v>69.45</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17">
       <c r="A36" t="s">
         <v>53</v>
       </c>
@@ -2440,7 +2450,7 @@
         <v>69.510000000000005</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17">
       <c r="A37" t="s">
         <v>54</v>
       </c>
@@ -2487,7 +2497,7 @@
         <v>42.27</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17">
       <c r="A38" t="s">
         <v>55</v>
       </c>
@@ -2534,7 +2544,7 @@
         <v>62.51</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17">
       <c r="A39" t="s">
         <v>56</v>
       </c>
@@ -2581,7 +2591,7 @@
         <v>63.27</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:17">
       <c r="A40" s="3" t="s">
         <v>57</v>
       </c>
@@ -2631,7 +2641,7 @@
         <v>162.65509030000001</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17">
       <c r="A41" s="3" t="s">
         <v>58</v>
       </c>
@@ -2681,7 +2691,7 @@
         <v>159.43121337890619</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17">
       <c r="A42" s="3" t="s">
         <v>59</v>
       </c>
@@ -2734,7 +2744,7 @@
         <v>178.8307189941406</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17">
       <c r="A43" s="3" t="s">
         <v>60</v>
       </c>
@@ -2787,7 +2797,7 @@
         <v>150.78038024902341</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17">
       <c r="A44" s="3" t="s">
         <v>61</v>
       </c>
@@ -2834,7 +2844,7 @@
         <v>71.7</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17">
       <c r="A45" s="3" t="s">
         <v>62</v>
       </c>
@@ -2881,7 +2891,7 @@
         <v>50.3</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17">
       <c r="A46" s="3" t="s">
         <v>63</v>
       </c>
@@ -2934,7 +2944,7 @@
         <v>62.698310852050781</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17">
       <c r="A47" s="3" t="s">
         <v>64</v>
       </c>
@@ -2987,7 +2997,7 @@
         <v>61.2</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17">
       <c r="A48" s="3" t="s">
         <v>65</v>
       </c>
@@ -3037,7 +3047,7 @@
         <v>61.2</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="s">
         <v>66</v>
       </c>
@@ -3087,7 +3097,7 @@
         <v>64.001168318171622</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19">
       <c r="A50" s="3" t="s">
         <v>67</v>
       </c>
@@ -3134,7 +3144,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19">
       <c r="A51" s="3" t="s">
         <v>68</v>
       </c>
@@ -3181,7 +3191,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19">
       <c r="A52" s="3" t="s">
         <v>69</v>
       </c>
@@ -3234,7 +3244,7 @@
         <v>0.12180000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19">
       <c r="A53" s="3" t="s">
         <v>70</v>
       </c>
@@ -3287,7 +3297,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19">
       <c r="A54" s="3" t="s">
         <v>71</v>
       </c>
@@ -3340,7 +3350,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19">
       <c r="A55" s="3" t="s">
         <v>72</v>
       </c>
@@ -3393,7 +3403,7 @@
         <v>0.126</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19">
       <c r="A56" s="3" t="s">
         <v>73</v>
       </c>
@@ -3446,7 +3456,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19">
       <c r="A57" s="3" t="s">
         <v>74</v>
       </c>
@@ -3499,7 +3509,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19">
       <c r="A58" s="3" t="s">
         <v>75</v>
       </c>
@@ -3555,7 +3565,7 @@
         <v>0.64400000000000002</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19">
       <c r="A59" s="3" t="s">
         <v>76</v>
       </c>
@@ -3611,7 +3621,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19">
       <c r="A60" s="3" t="s">
         <v>77</v>
       </c>
@@ -3667,7 +3677,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19">
       <c r="A61" s="3" t="s">
         <v>78</v>
       </c>
@@ -3724,7 +3734,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19">
       <c r="A62" s="3" t="s">
         <v>79</v>
       </c>
@@ -3781,7 +3791,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19">
       <c r="A63" s="3" t="s">
         <v>80</v>
       </c>
@@ -3838,7 +3848,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19">
       <c r="A64" s="3" t="s">
         <v>81</v>
       </c>
@@ -3895,7 +3905,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19">
       <c r="A65" s="3" t="s">
         <v>82</v>
       </c>
@@ -3951,7 +3961,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19">
       <c r="A66" s="3" t="s">
         <v>83</v>
       </c>
@@ -4007,7 +4017,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19">
       <c r="A67" s="3" t="s">
         <v>84</v>
       </c>
@@ -4063,7 +4073,7 @@
         <v>0.31900000000000001</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19">
       <c r="A68" s="3" t="s">
         <v>85</v>
       </c>
@@ -4119,7 +4129,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19">
       <c r="A69" s="3" t="s">
         <v>86</v>
       </c>
@@ -4176,7 +4186,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19">
       <c r="A70" s="3" t="s">
         <v>87</v>
       </c>
@@ -4233,7 +4243,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19">
       <c r="A71" s="3" t="s">
         <v>88</v>
       </c>
@@ -4290,7 +4300,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19">
       <c r="A72" s="3" t="s">
         <v>89</v>
       </c>
@@ -4347,7 +4357,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19">
       <c r="A73" s="3" t="s">
         <v>90</v>
       </c>
@@ -4403,7 +4413,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19">
       <c r="A74" s="3" t="s">
         <v>91</v>
       </c>
@@ -4459,7 +4469,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19">
       <c r="A75" s="3" t="s">
         <v>92</v>
       </c>
@@ -4515,7 +4525,7 @@
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19">
       <c r="A76" s="3" t="s">
         <v>93</v>
       </c>
@@ -4569,6 +4579,234 @@
       </c>
       <c r="S76" s="2">
         <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="77" spans="1:19">
+      <c r="A77" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B77" s="7">
+        <v>5</v>
+      </c>
+      <c r="C77" s="7">
+        <v>6</v>
+      </c>
+      <c r="D77" s="7">
+        <v>7</v>
+      </c>
+      <c r="E77" s="7">
+        <v>12</v>
+      </c>
+      <c r="F77" s="7">
+        <v>14</v>
+      </c>
+      <c r="G77" s="7">
+        <v>15</v>
+      </c>
+      <c r="H77" s="7">
+        <v>5</v>
+      </c>
+      <c r="I77" s="7">
+        <v>6</v>
+      </c>
+      <c r="J77" s="7">
+        <v>7</v>
+      </c>
+      <c r="K77" s="7">
+        <v>11</v>
+      </c>
+      <c r="L77" s="7">
+        <v>13</v>
+      </c>
+      <c r="M77" s="7">
+        <v>15</v>
+      </c>
+      <c r="N77" s="7">
+        <v>0</v>
+      </c>
+      <c r="O77" s="7"/>
+      <c r="P77" s="7">
+        <v>71.2</v>
+      </c>
+      <c r="Q77" s="2">
+        <v>78.09</v>
+      </c>
+      <c r="R77" s="2">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="S77" s="2">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="78" spans="1:19">
+      <c r="A78" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B78" s="7">
+        <v>5</v>
+      </c>
+      <c r="C78" s="7">
+        <v>6</v>
+      </c>
+      <c r="D78" s="7">
+        <v>8</v>
+      </c>
+      <c r="E78" s="7">
+        <v>11</v>
+      </c>
+      <c r="F78" s="7">
+        <v>15</v>
+      </c>
+      <c r="G78" s="7">
+        <v>16</v>
+      </c>
+      <c r="H78" s="7">
+        <v>5</v>
+      </c>
+      <c r="I78" s="7">
+        <v>6</v>
+      </c>
+      <c r="J78" s="7">
+        <v>8</v>
+      </c>
+      <c r="K78" s="7">
+        <v>11</v>
+      </c>
+      <c r="L78" s="7">
+        <v>13</v>
+      </c>
+      <c r="M78" s="7">
+        <v>16</v>
+      </c>
+      <c r="N78" s="7">
+        <v>0</v>
+      </c>
+      <c r="O78" s="7"/>
+      <c r="P78" s="7">
+        <v>71.2</v>
+      </c>
+      <c r="Q78" s="2">
+        <v>76.83</v>
+      </c>
+      <c r="R78" s="2">
+        <v>0.23</v>
+      </c>
+      <c r="S78" s="2">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="79" spans="1:19">
+      <c r="A79" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B79" s="7">
+        <v>5</v>
+      </c>
+      <c r="C79" s="7">
+        <v>6</v>
+      </c>
+      <c r="D79" s="7">
+        <v>7</v>
+      </c>
+      <c r="E79" s="7">
+        <v>8</v>
+      </c>
+      <c r="F79" s="7">
+        <v>9</v>
+      </c>
+      <c r="G79" s="7">
+        <v>12</v>
+      </c>
+      <c r="H79" s="7">
+        <v>5</v>
+      </c>
+      <c r="I79" s="7">
+        <v>6</v>
+      </c>
+      <c r="J79" s="7">
+        <v>7</v>
+      </c>
+      <c r="K79" s="7">
+        <v>8</v>
+      </c>
+      <c r="L79" s="7">
+        <v>9</v>
+      </c>
+      <c r="M79" s="7">
+        <v>10</v>
+      </c>
+      <c r="N79" s="7">
+        <v>0</v>
+      </c>
+      <c r="O79" s="7"/>
+      <c r="P79" s="7">
+        <v>64.400000000000006</v>
+      </c>
+      <c r="Q79" s="2">
+        <v>83.42</v>
+      </c>
+      <c r="R79" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="S79" s="2">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19">
+      <c r="A80" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B80" s="7">
+        <v>5</v>
+      </c>
+      <c r="C80" s="7">
+        <v>6</v>
+      </c>
+      <c r="D80" s="7">
+        <v>7</v>
+      </c>
+      <c r="E80" s="7">
+        <v>8</v>
+      </c>
+      <c r="F80" s="7">
+        <v>9</v>
+      </c>
+      <c r="G80" s="7">
+        <v>13</v>
+      </c>
+      <c r="H80" s="7">
+        <v>5</v>
+      </c>
+      <c r="I80" s="7">
+        <v>6</v>
+      </c>
+      <c r="J80" s="7">
+        <v>7</v>
+      </c>
+      <c r="K80" s="7">
+        <v>8</v>
+      </c>
+      <c r="L80" s="7">
+        <v>9</v>
+      </c>
+      <c r="M80" s="7">
+        <v>12</v>
+      </c>
+      <c r="N80" s="7">
+        <v>0</v>
+      </c>
+      <c r="O80" s="7"/>
+      <c r="P80" s="7">
+        <v>71.2</v>
+      </c>
+      <c r="Q80" s="2">
+        <v>79.760000000000005</v>
+      </c>
+      <c r="R80" s="2">
+        <v>0.32</v>
+      </c>
+      <c r="S80" s="2">
+        <v>0.47</v>
       </c>
     </row>
   </sheetData>
@@ -4580,13 +4818,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Z68"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4639,7 +4877,7 @@
         <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>18</v>
@@ -4652,7 +4890,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -4699,7 +4937,7 @@
         <v>59.02</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -4746,7 +4984,7 @@
         <v>57.46</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -4793,7 +5031,7 @@
         <v>58.23</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -4840,7 +5078,7 @@
         <v>58.23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -4887,7 +5125,7 @@
         <v>64.75</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -4934,7 +5172,7 @@
         <v>50.68</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -4981,7 +5219,7 @@
         <v>64.75</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -5028,7 +5266,7 @@
         <v>50.68</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -5075,7 +5313,7 @@
         <v>64.75</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -5122,7 +5360,7 @@
         <v>76.66</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -5169,7 +5407,7 @@
         <v>71.22</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -5216,7 +5454,7 @@
         <v>73.069999999999993</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -5263,7 +5501,7 @@
         <v>37.53</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -5310,7 +5548,7 @@
         <v>76.63</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -5357,7 +5595,7 @@
         <v>73.739999999999995</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -5404,7 +5642,7 @@
         <v>61.64</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -5451,7 +5689,7 @@
         <v>75.81</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -5498,7 +5736,7 @@
         <v>59.04</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -5545,7 +5783,7 @@
         <v>48.7</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -5592,7 +5830,7 @@
         <v>55.97</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -5639,7 +5877,7 @@
         <v>38.340000000000003</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -5686,7 +5924,7 @@
         <v>56.59</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16">
       <c r="A24" t="s">
         <v>41</v>
       </c>
@@ -5733,7 +5971,7 @@
         <v>69.42</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16">
       <c r="A25" t="s">
         <v>42</v>
       </c>
@@ -5780,7 +6018,7 @@
         <v>69.510000000000005</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -5827,7 +6065,7 @@
         <v>69.58</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16">
       <c r="A27" t="s">
         <v>44</v>
       </c>
@@ -5874,7 +6112,7 @@
         <v>54.39</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16">
       <c r="A28" t="s">
         <v>45</v>
       </c>
@@ -5921,7 +6159,7 @@
         <v>69.45</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16">
       <c r="A29" t="s">
         <v>46</v>
       </c>
@@ -5968,7 +6206,7 @@
         <v>69.510000000000005</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16">
       <c r="A30" t="s">
         <v>47</v>
       </c>
@@ -6015,7 +6253,7 @@
         <v>42.27</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -6062,7 +6300,7 @@
         <v>62.51</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16">
       <c r="A32" t="s">
         <v>49</v>
       </c>
@@ -6109,9 +6347,9 @@
         <v>63.27</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19">
       <c r="A33" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B33">
         <v>27</v>
@@ -6162,7 +6400,7 @@
         <v>81.815345764160156</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19">
       <c r="A34" s="2" t="s">
         <v>61</v>
       </c>
@@ -6215,7 +6453,7 @@
         <v>211.7365417480469</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19">
       <c r="A35" s="2" t="s">
         <v>62</v>
       </c>
@@ -6268,7 +6506,7 @@
         <v>209.16239929199219</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19">
       <c r="A36" s="2" t="s">
         <v>63</v>
       </c>
@@ -6315,7 +6553,7 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19">
       <c r="A37" s="2" t="s">
         <v>66</v>
       </c>
@@ -6368,7 +6606,7 @@
         <v>61.674495697021477</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19">
       <c r="A38" s="2" t="s">
         <v>67</v>
       </c>
@@ -6421,7 +6659,7 @@
         <v>58.28</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19">
       <c r="A39" s="3" t="s">
         <v>68</v>
       </c>
@@ -6471,7 +6709,7 @@
         <v>58.658827448472017</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19">
       <c r="A40" s="3" t="s">
         <v>69</v>
       </c>
@@ -6521,7 +6759,7 @@
         <v>58.658827087301148</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19">
       <c r="A41" s="3" t="s">
         <v>70</v>
       </c>
@@ -6574,7 +6812,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19">
       <c r="A42" s="3" t="s">
         <v>71</v>
       </c>
@@ -6627,7 +6865,7 @@
         <v>4.7699999999999999E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19">
       <c r="A43" s="3" t="s">
         <v>72</v>
       </c>
@@ -6677,7 +6915,7 @@
         <v>63.8</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19">
       <c r="A44" s="3" t="s">
         <v>73</v>
       </c>
@@ -6730,7 +6968,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19">
       <c r="A45" s="3" t="s">
         <v>74</v>
       </c>
@@ -6783,7 +7021,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19">
       <c r="A46" s="3" t="s">
         <v>75</v>
       </c>
@@ -6836,7 +7074,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19">
       <c r="A47" s="3" t="s">
         <v>76</v>
       </c>
@@ -6892,7 +7130,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19">
       <c r="A48" s="3" t="s">
         <v>77</v>
       </c>
@@ -6948,7 +7186,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19">
       <c r="A49" s="3" t="s">
         <v>78</v>
       </c>
@@ -7004,7 +7242,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19">
       <c r="A50" s="3" t="s">
         <v>79</v>
       </c>
@@ -7061,7 +7299,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19">
       <c r="A51" s="3" t="s">
         <v>80</v>
       </c>
@@ -7118,7 +7356,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19">
       <c r="A52" s="3" t="s">
         <v>81</v>
       </c>
@@ -7175,7 +7413,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19">
       <c r="A53" s="3" t="s">
         <v>82</v>
       </c>
@@ -7232,7 +7470,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19">
       <c r="A54" s="3" t="s">
         <v>83</v>
       </c>
@@ -7289,7 +7527,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19">
       <c r="A55" s="3" t="s">
         <v>84</v>
       </c>
@@ -7346,7 +7584,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19">
       <c r="A56" s="3" t="s">
         <v>85</v>
       </c>
@@ -7403,7 +7641,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19">
       <c r="A57" s="3" t="s">
         <v>86</v>
       </c>
@@ -7460,7 +7698,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19">
       <c r="A58" s="3" t="s">
         <v>87</v>
       </c>
@@ -7517,7 +7755,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19">
       <c r="A59" s="3" t="s">
         <v>88</v>
       </c>
@@ -7574,7 +7812,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19">
       <c r="A60" s="3" t="s">
         <v>89</v>
       </c>
@@ -7631,7 +7869,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19">
       <c r="A61" s="3" t="s">
         <v>90</v>
       </c>
@@ -7688,7 +7926,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19">
       <c r="A62" s="3" t="s">
         <v>91</v>
       </c>
@@ -7745,7 +7983,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19">
       <c r="A63" s="3" t="s">
         <v>92</v>
       </c>
@@ -7801,7 +8039,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19">
       <c r="A64" s="3" t="s">
         <v>93</v>
       </c>
@@ -7857,24 +8095,233 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A65" s="3"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
-      <c r="H65" s="2"/>
-      <c r="I65" s="2"/>
-      <c r="J65" s="2"/>
-      <c r="K65" s="2"/>
-      <c r="L65" s="2"/>
-      <c r="M65" s="2"/>
-      <c r="N65" s="2"/>
-      <c r="Q65" s="2"/>
-      <c r="R65" s="2"/>
-      <c r="S65" s="2"/>
+    <row r="65" spans="1:19">
+      <c r="A65" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B65" s="7">
+        <v>5</v>
+      </c>
+      <c r="C65" s="7">
+        <v>6</v>
+      </c>
+      <c r="D65" s="7">
+        <v>7</v>
+      </c>
+      <c r="E65" s="7">
+        <v>8</v>
+      </c>
+      <c r="F65" s="7">
+        <v>10</v>
+      </c>
+      <c r="G65" s="7">
+        <v>19</v>
+      </c>
+      <c r="H65" s="7">
+        <v>5</v>
+      </c>
+      <c r="I65" s="7">
+        <v>6</v>
+      </c>
+      <c r="J65" s="7">
+        <v>7</v>
+      </c>
+      <c r="K65" s="7">
+        <v>8</v>
+      </c>
+      <c r="L65" s="7">
+        <v>10</v>
+      </c>
+      <c r="M65" s="7">
+        <v>19</v>
+      </c>
+      <c r="N65" s="7">
+        <v>1</v>
+      </c>
+      <c r="O65" s="7"/>
+      <c r="P65" s="7">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="Q65" s="2">
+        <v>79.48</v>
+      </c>
+      <c r="R65" s="2">
+        <v>0.48</v>
+      </c>
+      <c r="S65" s="2">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19">
+      <c r="A66" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B66" s="7">
+        <v>5</v>
+      </c>
+      <c r="C66" s="7">
+        <v>6</v>
+      </c>
+      <c r="D66" s="7">
+        <v>14</v>
+      </c>
+      <c r="E66" s="7">
+        <v>16</v>
+      </c>
+      <c r="F66" s="7">
+        <v>34</v>
+      </c>
+      <c r="G66" s="7">
+        <v>35</v>
+      </c>
+      <c r="H66" s="7">
+        <v>5</v>
+      </c>
+      <c r="I66" s="7">
+        <v>6</v>
+      </c>
+      <c r="J66" s="7">
+        <v>7</v>
+      </c>
+      <c r="K66" s="7">
+        <v>16</v>
+      </c>
+      <c r="L66" s="7">
+        <v>20</v>
+      </c>
+      <c r="M66" s="7">
+        <v>35</v>
+      </c>
+      <c r="N66" s="7">
+        <v>1</v>
+      </c>
+      <c r="O66" s="7"/>
+      <c r="P66" s="7">
+        <v>69.599999999999994</v>
+      </c>
+      <c r="Q66" s="2">
+        <v>91.07</v>
+      </c>
+      <c r="R66" s="2">
+        <v>1.33</v>
+      </c>
+      <c r="S66" s="2">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19">
+      <c r="A67" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B67" s="7">
+        <v>7</v>
+      </c>
+      <c r="C67" s="7">
+        <v>8</v>
+      </c>
+      <c r="D67" s="7">
+        <v>10</v>
+      </c>
+      <c r="E67" s="7">
+        <v>14</v>
+      </c>
+      <c r="F67" s="7">
+        <v>15</v>
+      </c>
+      <c r="G67" s="7">
+        <v>26</v>
+      </c>
+      <c r="H67" s="7">
+        <v>7</v>
+      </c>
+      <c r="I67" s="7">
+        <v>8</v>
+      </c>
+      <c r="J67" s="7">
+        <v>9</v>
+      </c>
+      <c r="K67" s="7">
+        <v>14</v>
+      </c>
+      <c r="L67" s="7">
+        <v>15</v>
+      </c>
+      <c r="M67" s="7">
+        <v>17</v>
+      </c>
+      <c r="N67" s="7">
+        <v>1</v>
+      </c>
+      <c r="O67" s="7"/>
+      <c r="P67" s="7">
+        <v>66</v>
+      </c>
+      <c r="Q67" s="2">
+        <v>85.54</v>
+      </c>
+      <c r="R67" s="2">
+        <v>0.97</v>
+      </c>
+      <c r="S67" s="2">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="68" spans="1:19">
+      <c r="A68" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B68" s="7">
+        <v>5</v>
+      </c>
+      <c r="C68" s="7">
+        <v>6</v>
+      </c>
+      <c r="D68" s="7">
+        <v>10</v>
+      </c>
+      <c r="E68" s="7">
+        <v>11</v>
+      </c>
+      <c r="F68" s="7">
+        <v>12</v>
+      </c>
+      <c r="G68" s="7">
+        <v>16</v>
+      </c>
+      <c r="H68" s="7">
+        <v>5</v>
+      </c>
+      <c r="I68" s="7">
+        <v>6</v>
+      </c>
+      <c r="J68" s="7">
+        <v>7</v>
+      </c>
+      <c r="K68" s="7">
+        <v>11</v>
+      </c>
+      <c r="L68" s="7">
+        <v>12</v>
+      </c>
+      <c r="M68" s="7">
+        <v>14</v>
+      </c>
+      <c r="N68" s="7">
+        <v>1</v>
+      </c>
+      <c r="O68" s="7"/>
+      <c r="P68" s="7">
+        <v>58.9</v>
+      </c>
+      <c r="Q68" s="2">
+        <v>82.67</v>
+      </c>
+      <c r="R68" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="S68" s="2">
+        <v>0.45</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>